<commit_message>
Update email verification OTP test cases
</commit_message>
<xml_diff>
--- a/test_data/users.xlsx
+++ b/test_data/users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VIVI 2026\cex-automation\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C170F3D1-42BB-4EF5-B2F3-7A85F898FF01}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08372BEA-362E-43D9-AC16-D9B9B7431492}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="297">
   <si>
     <t>ID</t>
   </si>
@@ -1090,42 +1090,15 @@
     </r>
   </si>
   <si>
-    <t>REG_038</t>
-  </si>
-  <si>
-    <t>Verify OTP chỉ cho nhập số</t>
-  </si>
-  <si>
     <t>User ở màn hình verify email</t>
   </si>
   <si>
-    <t>abcdef</t>
-  </si>
-  <si>
-    <t>1. Nhập chữ vào OTP</t>
-  </si>
-  <si>
-    <t>Không cho nhập chữ hoặc hiển thị lỗi format</t>
-  </si>
-  <si>
     <t>REG_039</t>
   </si>
   <si>
-    <t>Verify nhập OTP dưới 6 số</t>
-  </si>
-  <si>
-    <t>1. Nhập 5 số</t>
-  </si>
-  <si>
     <t>REG_040</t>
   </si>
   <si>
-    <t>Verify nhập đủ 6 số thì button enabled</t>
-  </si>
-  <si>
-    <t>1. Nhập đủ 6 số OTP</t>
-  </si>
-  <si>
     <t>REG_041</t>
   </si>
   <si>
@@ -1273,25 +1246,10 @@
     <t>REG_048</t>
   </si>
   <si>
-    <t>Verify paste OTP 6 số</t>
-  </si>
-  <si>
-    <t>1. Copy OTP 6 số 2. Paste vào ô đầu tiên</t>
-  </si>
-  <si>
     <t>OTP được fill đủ 6 ô, button Tiếp theo enabled</t>
   </si>
   <si>
     <t>REG_049</t>
-  </si>
-  <si>
-    <t>Verify paste OTP quá 6 số</t>
-  </si>
-  <si>
-    <t>1. Paste chuỗi 9 số</t>
-  </si>
-  <si>
-    <t>Chỉ nhận 6 số đầu hoặc hiển thị lỗi theo rule hệ thống</t>
   </si>
   <si>
     <t>REG_050</t>
@@ -1521,6 +1479,42 @@
       </rPr>
       <t>Đăng ký</t>
     </r>
+  </si>
+  <si>
+    <t>Verify nhập OTP dưới 6 kí tự</t>
+  </si>
+  <si>
+    <t>Verify nhập đủ 6 kí tự thì button enabled</t>
+  </si>
+  <si>
+    <t>1. Nhập 5 kí tự cả số cả chữ</t>
+  </si>
+  <si>
+    <t>1. Nhập đủ 6 kí tự OTP</t>
+  </si>
+  <si>
+    <t>Verify paste OTP quá 6 kí tự</t>
+  </si>
+  <si>
+    <t>Verify paste OTP 6 kí tự</t>
+  </si>
+  <si>
+    <t>1. Copy OTP 6 kí tự 2. Paste vào ô đầu tiên</t>
+  </si>
+  <si>
+    <t>1. Paste chuỗi 9 kí tự</t>
+  </si>
+  <si>
+    <t>Chỉ nhận 6 kí tự đầu hoặc hiển thị lỗi theo rule hệ thống</t>
+  </si>
+  <si>
+    <t>1A3B5C</t>
+  </si>
+  <si>
+    <t>1A3B5C7D9</t>
+  </si>
+  <si>
+    <t>1A3B5</t>
   </si>
 </sst>
 </file>
@@ -1895,7 +1889,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="21" customWidth="1"/>
@@ -1954,7 +1948,7 @@
         <v>13</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>298</v>
+        <v>284</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>14</v>
@@ -2981,7 +2975,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="240">
+    <row r="38" spans="1:9" ht="45">
       <c r="A38" s="2" t="s">
         <v>174</v>
       </c>
@@ -3010,27 +3004,27 @@
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="90">
+    <row r="39" spans="1:9" ht="30">
       <c r="A39" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>180</v>
+        <v>285</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>182</v>
+        <v>296</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>183</v>
+        <v>287</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>184</v>
+        <v>27</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>15</v>
@@ -3039,27 +3033,27 @@
         <v>16</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="60">
+    <row r="40" spans="1:9" ht="30">
       <c r="A40" s="2" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>186</v>
+        <v>286</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E40" s="2">
-        <v>12345</v>
+        <v>179</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>294</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>187</v>
+        <v>288</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>15</v>
@@ -3068,114 +3062,114 @@
         <v>16</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="75">
+    <row r="41" spans="1:9" ht="150">
       <c r="A41" s="2" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C41" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="135">
+      <c r="A42" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E41" s="2">
-        <v>123456</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="150">
-      <c r="A42" s="2" t="s">
-        <v>191</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E42" s="2">
+        <v>0</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="H42" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="90">
+      <c r="A43" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="135">
-      <c r="A43" s="2" t="s">
-        <v>198</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C43" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="120">
+      <c r="A44" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E43" s="2">
-        <v>0</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="90">
-      <c r="A44" s="2" t="s">
-        <v>202</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>207</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>15</v>
@@ -3184,27 +3178,27 @@
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="120">
+    <row r="45" spans="1:9" ht="105">
       <c r="A45" s="2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>15</v>
@@ -3213,56 +3207,56 @@
         <v>16</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="105">
+    <row r="46" spans="1:9" ht="30">
       <c r="A46" s="2" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>13</v>
+        <v>294</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="90">
+    <row r="47" spans="1:9" ht="30">
       <c r="A47" s="2" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E47" s="2">
-        <v>123456</v>
+        <v>215</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>294</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>56</v>
@@ -3271,27 +3265,27 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="105">
+    <row r="48" spans="1:9" ht="30">
       <c r="A48" s="2" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>223</v>
+        <v>290</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="E48" s="2">
-        <v>123456</v>
+        <v>179</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>294</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>225</v>
+        <v>291</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>56</v>
@@ -3300,27 +3294,27 @@
         <v>16</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="105">
+    <row r="49" spans="1:9" ht="30">
       <c r="A49" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>228</v>
+        <v>289</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E49" s="2">
-        <v>123456</v>
+        <v>179</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>295</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>229</v>
+        <v>292</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>230</v>
+        <v>293</v>
       </c>
       <c r="H49" s="2" t="s">
         <v>56</v>
@@ -3329,27 +3323,27 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="105">
+    <row r="50" spans="1:9" ht="45">
       <c r="A50" s="2" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E50" s="2">
-        <v>123456789</v>
+        <v>179</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>233</v>
+        <v>135</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="H50" s="2" t="s">
         <v>56</v>
@@ -3358,328 +3352,299 @@
         <v>16</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="105">
+    <row r="51" spans="1:9" ht="315">
       <c r="A51" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="180">
+      <c r="A52" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C51" s="2" t="s">
+      <c r="G52" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="D51" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E51" s="2" t="s">
+      <c r="H52" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="225">
+      <c r="A53" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E53" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F51" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="H51" s="2" t="s">
+      <c r="F53" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="H53" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="I51" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" ht="315">
-      <c r="A52" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E52" s="2" t="s">
+      <c r="I53" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="135">
+      <c r="A54" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="F52" s="2" t="s">
+      <c r="B54" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="G52" s="2" t="s">
+      <c r="D54" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="H52" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="I52" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" ht="180">
-      <c r="A53" s="2" t="s">
+      <c r="E54" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="C53" s="2" t="s">
+      <c r="F54" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="D53" s="2" t="s">
+      <c r="G54" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="E53" s="2" t="s">
+      <c r="H54" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="150">
+      <c r="A55" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="F53" s="2" t="s">
+      <c r="B55" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="C55" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="H53" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="I53" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" ht="225">
-      <c r="A54" s="2" t="s">
+      <c r="D55" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="C54" s="2" t="s">
+      <c r="E55" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="F55" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="E54" s="2" t="s">
+      <c r="G55" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="120">
+      <c r="A56" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E56" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F54" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="G54" s="2" t="s">
+      <c r="F56" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I56" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="H54" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="I54" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" ht="135">
-      <c r="A55" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="F55" s="2" t="s">
+    </row>
+    <row r="57" spans="1:9" ht="105">
+      <c r="A57" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="G55" s="2" t="s">
+      <c r="B57" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="H55" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="I55" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="150">
-      <c r="A56" s="2" t="s">
+      <c r="D57" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E57" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="F57" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="G57" s="2" t="s">
         <v>264</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="H56" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="I56" s="2" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" ht="120">
-      <c r="A57" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>273</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I57" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="120">
+      <c r="A58" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="F58" s="2" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" ht="105">
-      <c r="A58" s="2" t="s">
+      <c r="G58" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="105">
+      <c r="A59" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E59" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="C58" s="2" t="s">
+      <c r="F59" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D58" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E58" s="2" t="s">
+      <c r="G59" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="F58" s="2" t="s">
+      <c r="H59" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="120">
+      <c r="A60" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="G58" s="2" t="s">
+      <c r="B60" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="H58" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="120">
-      <c r="A59" s="2" t="s">
+      <c r="C60" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="B59" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="C59" s="2" t="s">
+      <c r="D60" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="D59" s="2" t="s">
+      <c r="E60" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="E59" s="4" t="s">
+      <c r="G60" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F59" s="2" t="s">
+      <c r="H60" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9">
+      <c r="A62" t="s">
         <v>283</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="H59" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="I59" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="105">
-      <c r="A60" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="E60" s="4" t="s">
-        <v>288</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" ht="120">
-      <c r="A61" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="G61" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="I61" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9">
-      <c r="A63" t="s">
-        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>